<commit_message>
v13: carros con las reglas de W-CAR y la demanda 2035, banda sur compacta y rótulos sin pisar equipos
Lugares de carros: 317 en lugar de 550 (despacho 84, pintados 49, sala de pérdidas 17,
retenidos 74, liberados 70, rechazados 23) con el mes pico de 2035 de X-CAR; reservas
RV-C1 a RV-C3, entrada de cilindros C-16A, flujos y corte A-A por y = 6,0 m. Franjas sin
uso unidas a C-03, C-05, C-06 y C-10.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/v10/Layout_v10_zonas_y_equipos.xlsx
+++ b/salida/v10/Layout_v10_zonas_y_equipos.xlsx
@@ -579,10 +579,10 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>736.1</v>
+        <v>691.1</v>
       </c>
       <c r="C9" s="5" t="n">
-        <v>20.6</v>
+        <v>19.3</v>
       </c>
     </row>
     <row r="10">
@@ -592,10 +592,10 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>248.4</v>
+        <v>205.5</v>
       </c>
       <c r="C10" s="5" t="n">
-        <v>7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="11">
@@ -618,10 +618,10 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>238.9</v>
+        <v>326.8</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>6.7</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="13">
@@ -2895,7 +2895,7 @@
         </is>
       </c>
       <c r="E45" s="5" t="n">
-        <v>21.8</v>
+        <v>21.3</v>
       </c>
       <c r="F45" s="5" t="n">
         <v>20</v>
@@ -2907,13 +2907,13 @@
         <v>25</v>
       </c>
       <c r="I45" s="5" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="J45" s="5" t="n">
         <v>5</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>35</v>
+        <v>37.5</v>
       </c>
       <c r="L45" s="4" t="n">
         <v>35</v>
@@ -2980,12 +2980,12 @@
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>C-03W</t>
+          <t>C-03E</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
         <is>
-          <t>Franja entre el corte y el cilindrado</t>
+          <t>Paso de los carros del marcado al cilindrado</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -2999,42 +2999,46 @@
         </is>
       </c>
       <c r="E47" s="5" t="n">
-        <v>21.3</v>
+        <v>24.8</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>20</v>
+        <v>26.4</v>
       </c>
       <c r="G47" s="5" t="n">
-        <v>21.8</v>
+        <v>28.8</v>
       </c>
       <c r="H47" s="5" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I47" s="5" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>5</v>
+        <v>2.6</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>2.5</v>
+        <v>10.4</v>
       </c>
       <c r="L47" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M47" s="4" t="inlineStr"/>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>W-CAR 2.1: los carros llenos esperan al costado de la mesa de marcado</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>C-03E</t>
+          <t>C-05</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>Paso de los carros del marcado al cilindrado</t>
+          <t>5 Soldadura longitudinal</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3048,46 +3052,44 @@
         </is>
       </c>
       <c r="E48" s="5" t="n">
-        <v>24.8</v>
+        <v>29.3</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>26.4</v>
+        <v>20</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>28.8</v>
+        <v>35.3</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="I48" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J48" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="J48" s="5" t="n">
-        <v>2.6</v>
-      </c>
       <c r="K48" s="5" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>22</v>
       </c>
       <c r="M48" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 2.1: los carros llenos esperan al costado de la mesa de marcado</t>
+          <t>W-CAR, tabla de espacios del puesto 5: ≈ 5,5 × 4,0 m</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>C-05</t>
+          <t>C-04</t>
         </is>
       </c>
       <c r="B49" s="4" t="inlineStr">
         <is>
-          <t>5 Soldadura longitudinal</t>
+          <t>4 Punteo del cuerpo</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3104,41 +3106,41 @@
         <v>29.3</v>
       </c>
       <c r="F49" s="5" t="n">
-        <v>20</v>
+        <v>24.5</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>34.8</v>
+        <v>35.3</v>
       </c>
       <c r="H49" s="5" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I49" s="5" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K49" s="5" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="L49" s="4" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="M49" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 5: ≈ 5,5 × 4,0 m</t>
+          <t>W-CAR, tabla de espacios del puesto 4: ≈ 6,0 × 4,5 m</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>C-04</t>
+          <t>C-45</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>4 Punteo del cuerpo</t>
+          <t>Cortina de soldadura entre 3 y 4/5</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
@@ -3152,44 +3154,46 @@
         </is>
       </c>
       <c r="E50" s="5" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="F50" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G50" s="5" t="n">
         <v>29.3</v>
-      </c>
-      <c r="F50" s="5" t="n">
-        <v>24.5</v>
-      </c>
-      <c r="G50" s="5" t="n">
-        <v>35.3</v>
       </c>
       <c r="H50" s="5" t="n">
         <v>29</v>
       </c>
       <c r="I50" s="5" t="n">
-        <v>6</v>
+        <v>0.5</v>
       </c>
       <c r="J50" s="5" t="n">
+        <v>9</v>
+      </c>
+      <c r="K50" s="5" t="n">
         <v>4.5</v>
       </c>
-      <c r="K50" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="L50" s="4" t="n">
-        <v>27</v>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M50" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 4: ≈ 6,0 × 4,5 m</t>
+          <t>W-CAR 4: cortina de soldadura</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>C-45</t>
+          <t>C-45b</t>
         </is>
       </c>
       <c r="B51" s="4" t="inlineStr">
         <is>
-          <t>Cortina de soldadura entre 3 y 4/5</t>
+          <t>Cortina de soldadura entre 4 y 5</t>
         </is>
       </c>
       <c r="C51" s="4" t="inlineStr">
@@ -3203,25 +3207,25 @@
         </is>
       </c>
       <c r="E51" s="5" t="n">
-        <v>28.8</v>
+        <v>29.3</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="G51" s="5" t="n">
-        <v>29.3</v>
+        <v>35.3</v>
       </c>
       <c r="H51" s="5" t="n">
-        <v>29</v>
+        <v>24.5</v>
       </c>
       <c r="I51" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="J51" s="5" t="n">
         <v>0.5</v>
       </c>
-      <c r="J51" s="5" t="n">
-        <v>9</v>
-      </c>
       <c r="K51" s="5" t="n">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="L51" s="4" t="inlineStr">
         <is>
@@ -3237,12 +3241,12 @@
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>C-45b</t>
+          <t>C-07</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>Cortina de soldadura entre 4 y 5</t>
+          <t>7 Armado y soldadura circunferencial</t>
         </is>
       </c>
       <c r="C52" s="4" t="inlineStr">
@@ -3256,13 +3260,13 @@
         </is>
       </c>
       <c r="E52" s="5" t="n">
-        <v>29.3</v>
+        <v>36.8</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G52" s="5" t="n">
-        <v>35.3</v>
+        <v>42.8</v>
       </c>
       <c r="H52" s="5" t="n">
         <v>24.5</v>
@@ -3271,31 +3275,29 @@
         <v>6</v>
       </c>
       <c r="J52" s="5" t="n">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="K52" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="L52" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>27</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>27</v>
       </c>
       <c r="M52" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 4: cortina de soldadura</t>
+          <t>W-CAR, tabla de espacios del puesto 7: ≈ 6,0 × 4,5 m</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>C-45c</t>
+          <t>C-06</t>
         </is>
       </c>
       <c r="B53" s="4" t="inlineStr">
         <is>
-          <t>Franja al este de la soldadura longitudinal</t>
+          <t>6 Soldadura de cupla en la cúpula</t>
         </is>
       </c>
       <c r="C53" s="4" t="inlineStr">
@@ -3309,42 +3311,44 @@
         </is>
       </c>
       <c r="E53" s="5" t="n">
-        <v>34.8</v>
+        <v>36.8</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>20</v>
+        <v>25.5</v>
       </c>
       <c r="G53" s="5" t="n">
-        <v>35.3</v>
+        <v>42.8</v>
       </c>
       <c r="H53" s="5" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I53" s="5" t="n">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="L53" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M53" s="4" t="inlineStr"/>
+        <v>21</v>
+      </c>
+      <c r="L53" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="M53" s="4" t="inlineStr">
+        <is>
+          <t>W-CAR, tabla de espacios del puesto 6: ≈ 4,5 × 3,5 m</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>C-07</t>
+          <t>C-67</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>7 Armado y soldadura circunferencial</t>
+          <t>Paso del carro canasto de cúpulas de 6 a 7</t>
         </is>
       </c>
       <c r="C54" s="4" t="inlineStr">
@@ -3361,41 +3365,43 @@
         <v>36.8</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>20</v>
+        <v>24.5</v>
       </c>
       <c r="G54" s="5" t="n">
         <v>42.8</v>
       </c>
       <c r="H54" s="5" t="n">
-        <v>24.5</v>
+        <v>25.5</v>
       </c>
       <c r="I54" s="5" t="n">
         <v>6</v>
       </c>
       <c r="J54" s="5" t="n">
-        <v>4.5</v>
+        <v>1</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>27</v>
-      </c>
-      <c r="L54" s="4" t="n">
-        <v>27</v>
+        <v>6</v>
+      </c>
+      <c r="L54" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M54" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 7: ≈ 6,0 × 4,5 m</t>
+          <t>W-CAR 6 y 7</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>C-06</t>
+          <t>C-08</t>
         </is>
       </c>
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>6 Soldadura de cupla en la cúpula</t>
+          <t>8 Soldadura de accesorios</t>
         </is>
       </c>
       <c r="C55" s="4" t="inlineStr">
@@ -3409,44 +3415,44 @@
         </is>
       </c>
       <c r="E55" s="5" t="n">
-        <v>36.8</v>
+        <v>43.3</v>
       </c>
       <c r="F55" s="5" t="n">
-        <v>25.5</v>
+        <v>20</v>
       </c>
       <c r="G55" s="5" t="n">
-        <v>41.3</v>
+        <v>49.8</v>
       </c>
       <c r="H55" s="5" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="I55" s="5" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="J55" s="5" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="K55" s="5" t="n">
+        <v>29.25</v>
+      </c>
+      <c r="L55" s="4" t="n">
         <v>29</v>
       </c>
-      <c r="I55" s="5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="J55" s="5" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="K55" s="5" t="n">
-        <v>15.75</v>
-      </c>
-      <c r="L55" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="M55" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 6: ≈ 4,5 × 3,5 m</t>
+          <t>W-CAR, tabla de espacios del puesto 8: ≈ 6,5 × 4,5 m</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>C-67</t>
+          <t>C-081</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>Paso del carro canasto de cúpulas de 6 a 7</t>
+          <t>8.1 Fabricación de accesorios</t>
         </is>
       </c>
       <c r="C56" s="4" t="inlineStr">
@@ -3460,46 +3466,44 @@
         </is>
       </c>
       <c r="E56" s="5" t="n">
-        <v>36.8</v>
+        <v>43.3</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="G56" s="5" t="n">
-        <v>42.8</v>
+        <v>51.3</v>
       </c>
       <c r="H56" s="5" t="n">
-        <v>25.5</v>
+        <v>29</v>
       </c>
       <c r="I56" s="5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J56" s="5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K56" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="L56" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>32</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="M56" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 6 y 7</t>
+          <t>W-CAR, tabla de espacios del puesto 8.1: ≈ 8,0 × 4,0 m</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>C-67b</t>
+          <t>C-78</t>
         </is>
       </c>
       <c r="B57" s="4" t="inlineStr">
         <is>
-          <t>Franja al este de la cupla</t>
+          <t>Cortina de soldadura entre 7 y 8</t>
         </is>
       </c>
       <c r="C57" s="4" t="inlineStr">
@@ -3513,42 +3517,46 @@
         </is>
       </c>
       <c r="E57" s="5" t="n">
-        <v>41.3</v>
+        <v>42.8</v>
       </c>
       <c r="F57" s="5" t="n">
-        <v>25.5</v>
+        <v>20</v>
       </c>
       <c r="G57" s="5" t="n">
-        <v>42.8</v>
+        <v>43.3</v>
       </c>
       <c r="H57" s="5" t="n">
         <v>29</v>
       </c>
       <c r="I57" s="5" t="n">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="J57" s="5" t="n">
-        <v>3.5</v>
+        <v>9</v>
       </c>
       <c r="K57" s="5" t="n">
-        <v>5.25</v>
+        <v>4.5</v>
       </c>
       <c r="L57" s="4" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="M57" s="4" t="inlineStr"/>
+      <c r="M57" s="4" t="inlineStr">
+        <is>
+          <t>W-CAR 8: cortina de soldadura</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>C-08</t>
+          <t>C-88</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>8 Soldadura de accesorios</t>
+          <t>Cortina entre 8 y 8.1</t>
         </is>
       </c>
       <c r="C58" s="4" t="inlineStr">
@@ -3565,41 +3573,43 @@
         <v>43.3</v>
       </c>
       <c r="F58" s="5" t="n">
-        <v>20</v>
+        <v>24.5</v>
       </c>
       <c r="G58" s="5" t="n">
-        <v>49.8</v>
+        <v>51.3</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="I58" s="5" t="n">
-        <v>6.5</v>
+        <v>8</v>
       </c>
       <c r="J58" s="5" t="n">
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="K58" s="5" t="n">
-        <v>29.25</v>
-      </c>
-      <c r="L58" s="4" t="n">
-        <v>29</v>
+        <v>4</v>
+      </c>
+      <c r="L58" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M58" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 8: ≈ 6,5 × 4,5 m</t>
+          <t>W-CAR 8: cortina de soldadura</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>C-081</t>
+          <t>C-08E</t>
         </is>
       </c>
       <c r="B59" s="4" t="inlineStr">
         <is>
-          <t>8.1 Fabricación de accesorios</t>
+          <t>Salida de los carros sobre su juego provisorio</t>
         </is>
       </c>
       <c r="C59" s="4" t="inlineStr">
@@ -3613,44 +3623,46 @@
         </is>
       </c>
       <c r="E59" s="5" t="n">
-        <v>43.3</v>
+        <v>49.8</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="G59" s="5" t="n">
         <v>51.3</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>29</v>
+        <v>24.5</v>
       </c>
       <c r="I59" s="5" t="n">
-        <v>8</v>
+        <v>1.5</v>
       </c>
       <c r="J59" s="5" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>32</v>
-      </c>
-      <c r="L59" s="4" t="n">
-        <v>32</v>
+        <v>6.75</v>
+      </c>
+      <c r="L59" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M59" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 8.1: ≈ 8,0 × 4,0 m</t>
+          <t>W-CAR 8: salida demarcada en amarillo</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>C-78</t>
+          <t>C-10</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>Cortina de soldadura entre 7 y 8</t>
+          <t>10 Secado</t>
         </is>
       </c>
       <c r="C60" s="4" t="inlineStr">
@@ -3664,46 +3676,44 @@
         </is>
       </c>
       <c r="E60" s="5" t="n">
-        <v>42.8</v>
+        <v>51.3</v>
       </c>
       <c r="F60" s="5" t="n">
         <v>20</v>
       </c>
       <c r="G60" s="5" t="n">
-        <v>43.3</v>
+        <v>54.8</v>
       </c>
       <c r="H60" s="5" t="n">
-        <v>29</v>
+        <v>22.5</v>
       </c>
       <c r="I60" s="5" t="n">
-        <v>0.5</v>
+        <v>3.5</v>
       </c>
       <c r="J60" s="5" t="n">
-        <v>9</v>
+        <v>2.5</v>
       </c>
       <c r="K60" s="5" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="L60" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>8.75</v>
+      </c>
+      <c r="L60" s="5" t="n">
+        <v>7.5</v>
       </c>
       <c r="M60" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 8: cortina de soldadura</t>
+          <t>W-CAR, tabla de espacios del puesto 10: ≈ 3,0 × 2,5 m</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>C-88</t>
+          <t>C-09</t>
         </is>
       </c>
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>Cortina entre 8 y 8.1</t>
+          <t>9 Prueba hidráulica</t>
         </is>
       </c>
       <c r="C61" s="4" t="inlineStr">
@@ -3717,46 +3727,44 @@
         </is>
       </c>
       <c r="E61" s="5" t="n">
-        <v>43.3</v>
+        <v>51.3</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="G61" s="5" t="n">
-        <v>51.3</v>
+        <v>57.3</v>
       </c>
       <c r="H61" s="5" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I61" s="5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J61" s="5" t="n">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="L61" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="L61" s="4" t="n">
+        <v>22</v>
       </c>
       <c r="M61" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 8: cortina de soldadura</t>
+          <t>W-CAR, tabla de espacios del puesto 9: ≈ 5,5 × 4,0 m</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>C-08E</t>
+          <t>C-910a</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Salida de los carros sobre su juego provisorio</t>
+          <t>Paso de la prueba hidráulica al secado</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -3770,25 +3778,25 @@
         </is>
       </c>
       <c r="E62" s="5" t="n">
-        <v>49.8</v>
+        <v>51.3</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>20</v>
+        <v>22.5</v>
       </c>
       <c r="G62" s="5" t="n">
-        <v>51.3</v>
+        <v>57.3</v>
       </c>
       <c r="H62" s="5" t="n">
-        <v>24.5</v>
+        <v>25</v>
       </c>
       <c r="I62" s="5" t="n">
-        <v>1.5</v>
+        <v>6</v>
       </c>
       <c r="J62" s="5" t="n">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="K62" s="5" t="n">
-        <v>6.75</v>
+        <v>15</v>
       </c>
       <c r="L62" s="4" t="inlineStr">
         <is>
@@ -3797,19 +3805,19 @@
       </c>
       <c r="M62" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 8: salida demarcada en amarillo</t>
+          <t>W-CAR 9 y 10</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>C-10</t>
+          <t>C-910c</t>
         </is>
       </c>
       <c r="B63" s="4" t="inlineStr">
         <is>
-          <t>10 Secado</t>
+          <t>Salida del secado hacia el pulmón de despacho</t>
         </is>
       </c>
       <c r="C63" s="4" t="inlineStr">
@@ -3823,49 +3831,51 @@
         </is>
       </c>
       <c r="E63" s="5" t="n">
-        <v>51.8</v>
+        <v>54.8</v>
       </c>
       <c r="F63" s="5" t="n">
         <v>20</v>
       </c>
       <c r="G63" s="5" t="n">
-        <v>54.8</v>
+        <v>57.3</v>
       </c>
       <c r="H63" s="5" t="n">
         <v>22.5</v>
       </c>
       <c r="I63" s="5" t="n">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J63" s="5" t="n">
         <v>2.5</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>7.5</v>
-      </c>
-      <c r="L63" s="5" t="n">
-        <v>7.5</v>
+        <v>6.25</v>
+      </c>
+      <c r="L63" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M63" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 10: ≈ 3,0 × 2,5 m</t>
+          <t>W-CAR 10: los carros secos van al puesto 11, al otro lado del pasillo</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>C-09</t>
+          <t>M-04</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>9 Prueba hidráulica</t>
+          <t>4 Corte de disco y embutido (desbobinador, alimentador y prensa)</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Manuales 1 a 10 kg</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -3874,49 +3884,49 @@
         </is>
       </c>
       <c r="E64" s="5" t="n">
-        <v>51.3</v>
+        <v>15.4</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="G64" s="5" t="n">
-        <v>57.3</v>
+        <v>25.4</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>29</v>
+        <v>45</v>
       </c>
       <c r="I64" s="5" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="J64" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>24</v>
-      </c>
-      <c r="L64" s="4" t="n">
-        <v>22</v>
+        <v>40</v>
+      </c>
+      <c r="L64" s="5" t="n">
+        <v>26</v>
       </c>
       <c r="M64" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 9: ≈ 5,5 × 4,0 m</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>C-910a</t>
+          <t>M-PCU</t>
         </is>
       </c>
       <c r="B65" s="4" t="inlineStr">
         <is>
-          <t>Paso de la prueba hidráulica al secado</t>
+          <t>Zona de cúpulas (5 carros de 12 cajones), al lado del numerado</t>
         </is>
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Manuales 1 a 10 kg</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -3925,25 +3935,25 @@
         </is>
       </c>
       <c r="E65" s="5" t="n">
-        <v>51.3</v>
+        <v>25.4</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>22.5</v>
+        <v>41</v>
       </c>
       <c r="G65" s="5" t="n">
-        <v>57.3</v>
+        <v>28.3</v>
       </c>
       <c r="H65" s="5" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="I65" s="5" t="n">
-        <v>6</v>
+        <v>2.9</v>
       </c>
       <c r="J65" s="5" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="K65" s="5" t="n">
-        <v>15</v>
+        <v>11.6</v>
       </c>
       <c r="L65" s="4" t="inlineStr">
         <is>
@@ -3952,24 +3962,24 @@
       </c>
       <c r="M65" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 9 y 10</t>
+          <t>W-MAN 3: 3 a 5 carros, al lado del numerado y la soldadura de cuello</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>C-910b</t>
+          <t>M-06</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Franja junto al secado (lado oeste)</t>
+          <t>6 Numerado de cúpula (pegado a la soldadura de cuello)</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Manuales 1 a 10 kg</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -3978,47 +3988,49 @@
         </is>
       </c>
       <c r="E66" s="5" t="n">
-        <v>51.3</v>
+        <v>28.3</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="G66" s="5" t="n">
-        <v>51.8</v>
+        <v>30.9</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>22.5</v>
+        <v>45</v>
       </c>
       <c r="I66" s="5" t="n">
-        <v>0.5</v>
+        <v>2.6</v>
       </c>
       <c r="J66" s="5" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>1.25</v>
-      </c>
-      <c r="L66" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M66" s="4" t="inlineStr"/>
+        <v>10.4</v>
+      </c>
+      <c r="L66" s="5" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="M66" s="4" t="inlineStr">
+        <is>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 6: la cúpula pasa a mano a la soldadura de cuello de al lado</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>C-910c</t>
+          <t>M-07</t>
         </is>
       </c>
       <c r="B67" s="4" t="inlineStr">
         <is>
-          <t>Salida del secado hacia el pulmón de despacho</t>
+          <t>7 Soldadura del cuello a la cúpula</t>
         </is>
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Manuales 1 a 10 kg</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -4027,46 +4039,44 @@
         </is>
       </c>
       <c r="E67" s="5" t="n">
-        <v>54.8</v>
+        <v>30.9</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="G67" s="5" t="n">
-        <v>57.3</v>
+        <v>33.4</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>22.5</v>
+        <v>45</v>
       </c>
       <c r="I67" s="5" t="n">
         <v>2.5</v>
       </c>
       <c r="J67" s="5" t="n">
-        <v>2.5</v>
+        <v>4</v>
       </c>
       <c r="K67" s="5" t="n">
-        <v>6.25</v>
-      </c>
-      <c r="L67" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="L67" s="5" t="n">
+        <v>5.3</v>
       </c>
       <c r="M67" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 10: los carros secos van al puesto 11, al otro lado del pasillo</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>M-04</t>
+          <t>M-05</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>4 Corte de disco y embutido (desbobinador, alimentador y prensa)</t>
+          <t>5 Preparación de cuello (2 prensas de banco)</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -4080,28 +4090,28 @@
         </is>
       </c>
       <c r="E68" s="5" t="n">
-        <v>15.4</v>
+        <v>33.4</v>
       </c>
       <c r="F68" s="5" t="n">
         <v>41</v>
       </c>
       <c r="G68" s="5" t="n">
-        <v>25.4</v>
+        <v>35.3</v>
       </c>
       <c r="H68" s="5" t="n">
         <v>45</v>
       </c>
       <c r="I68" s="5" t="n">
-        <v>10</v>
+        <v>1.9</v>
       </c>
       <c r="J68" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>40</v>
+        <v>7.6</v>
       </c>
       <c r="L68" s="5" t="n">
-        <v>26</v>
+        <v>4.5</v>
       </c>
       <c r="M68" s="4" t="inlineStr">
         <is>
@@ -4112,12 +4122,12 @@
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>M-PCU</t>
+          <t>M-03</t>
         </is>
       </c>
       <c r="B69" s="4" t="inlineStr">
         <is>
-          <t>Zona de cúpulas (5 carros de 12 cajones), al lado del numerado</t>
+          <t>3 Corte de tubo 1 kg (láser Leapion, orientado norte-sur)</t>
         </is>
       </c>
       <c r="C69" s="4" t="inlineStr">
@@ -4131,46 +4141,44 @@
         </is>
       </c>
       <c r="E69" s="5" t="n">
-        <v>25.4</v>
+        <v>15.4</v>
       </c>
       <c r="F69" s="5" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="G69" s="5" t="n">
+        <v>18</v>
+      </c>
+      <c r="H69" s="5" t="n">
         <v>41</v>
       </c>
-      <c r="G69" s="5" t="n">
-        <v>28.3</v>
-      </c>
-      <c r="H69" s="5" t="n">
-        <v>45</v>
-      </c>
       <c r="I69" s="5" t="n">
-        <v>2.9</v>
+        <v>2.6</v>
       </c>
       <c r="J69" s="5" t="n">
-        <v>4</v>
+        <v>13.6</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="L69" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>35.36</v>
+      </c>
+      <c r="L69" s="5" t="n">
+        <v>25.5</v>
       </c>
       <c r="M69" s="4" t="inlineStr">
         <is>
-          <t>W-MAN 3: 3 a 5 carros, al lado del numerado y la soldadura de cuello</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>M-06</t>
+          <t>M-PT</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>6 Numerado de cúpula (pegado a la soldadura de cuello)</t>
+          <t>Tramos 1 kg: carros «en consumo» y «lleno» al lado del encastre</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -4184,44 +4192,46 @@
         </is>
       </c>
       <c r="E70" s="5" t="n">
-        <v>28.3</v>
+        <v>18</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G70" s="5" t="n">
-        <v>30.9</v>
+        <v>21</v>
       </c>
       <c r="H70" s="5" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I70" s="5" t="n">
-        <v>2.6</v>
+        <v>3</v>
       </c>
       <c r="J70" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>10.4</v>
-      </c>
-      <c r="L70" s="5" t="n">
-        <v>2.3</v>
+        <v>12</v>
+      </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M70" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 6: la cúpula pasa a mano a la soldadura de cuello de al lado</t>
+          <t>W-MAN 2: al lado del encastre se demarcan dos posiciones de carro de 1,2 × 0,8 m, «en consumo» y «lleno»</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>M-07</t>
+          <t>M-10</t>
         </is>
       </c>
       <c r="B71" s="4" t="inlineStr">
         <is>
-          <t>7 Soldadura del cuello a la cúpula</t>
+          <t>10 Encastre de fondo y zona de fondos (5 carros)</t>
         </is>
       </c>
       <c r="C71" s="4" t="inlineStr">
@@ -4235,44 +4245,44 @@
         </is>
       </c>
       <c r="E71" s="5" t="n">
-        <v>30.9</v>
+        <v>21</v>
       </c>
       <c r="F71" s="5" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G71" s="5" t="n">
-        <v>33.4</v>
+        <v>26.6</v>
       </c>
       <c r="H71" s="5" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I71" s="5" t="n">
-        <v>2.5</v>
+        <v>5.6</v>
       </c>
       <c r="J71" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K71" s="5" t="n">
-        <v>10</v>
+        <v>22.4</v>
       </c>
       <c r="L71" s="5" t="n">
-        <v>5.3</v>
+        <v>3.6</v>
       </c>
       <c r="M71" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 3</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>M-05</t>
+          <t>M-11</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>5 Preparación de cuello (2 prensas de banco)</t>
+          <t>11 Bordoneado</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -4286,28 +4296,28 @@
         </is>
       </c>
       <c r="E72" s="5" t="n">
-        <v>33.4</v>
+        <v>26.6</v>
       </c>
       <c r="F72" s="5" t="n">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="G72" s="5" t="n">
-        <v>35.3</v>
+        <v>31</v>
       </c>
       <c r="H72" s="5" t="n">
-        <v>45</v>
+        <v>39</v>
       </c>
       <c r="I72" s="5" t="n">
-        <v>1.9</v>
+        <v>4.4</v>
       </c>
       <c r="J72" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K72" s="5" t="n">
-        <v>7.6</v>
+        <v>17.6</v>
       </c>
       <c r="L72" s="5" t="n">
-        <v>4.5</v>
+        <v>3.6</v>
       </c>
       <c r="M72" s="4" t="inlineStr">
         <is>
@@ -4318,12 +4328,12 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>M-03</t>
+          <t>M-PB</t>
         </is>
       </c>
       <c r="B73" s="4" t="inlineStr">
         <is>
-          <t>3 Corte de tubo 1 kg (láser Leapion, orientado norte-sur)</t>
+          <t>Pulmones del bordoneado a la soldadura circunferencial</t>
         </is>
       </c>
       <c r="C73" s="4" t="inlineStr">
@@ -4337,44 +4347,46 @@
         </is>
       </c>
       <c r="E73" s="5" t="n">
-        <v>15.4</v>
+        <v>31</v>
       </c>
       <c r="F73" s="5" t="n">
-        <v>27.4</v>
+        <v>35</v>
       </c>
       <c r="G73" s="5" t="n">
-        <v>18</v>
+        <v>35.3</v>
       </c>
       <c r="H73" s="5" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="I73" s="5" t="n">
-        <v>2.6</v>
+        <v>4.3</v>
       </c>
       <c r="J73" s="5" t="n">
-        <v>13.6</v>
+        <v>4</v>
       </c>
       <c r="K73" s="5" t="n">
-        <v>35.36</v>
-      </c>
-      <c r="L73" s="5" t="n">
-        <v>25.5</v>
+        <v>17.2</v>
+      </c>
+      <c r="L73" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M73" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>W-MAN 9 y 10</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>M-PT</t>
+          <t>M-08</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>Tramos 1 kg: carros «en consumo» y «lleno» al lado del encastre</t>
+          <t>8 Cilindrado</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -4391,43 +4403,41 @@
         <v>18</v>
       </c>
       <c r="F74" s="5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G74" s="5" t="n">
-        <v>21</v>
+        <v>23.4</v>
       </c>
       <c r="H74" s="5" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I74" s="5" t="n">
-        <v>3</v>
+        <v>5.4</v>
       </c>
       <c r="J74" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K74" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="L74" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>21.6</v>
+      </c>
+      <c r="L74" s="5" t="n">
+        <v>7.3</v>
       </c>
       <c r="M74" s="4" t="inlineStr">
         <is>
-          <t>W-MAN 2: al lado del encastre se demarcan dos posiciones de carro de 1,2 × 0,8 m, «en consumo» y «lleno»</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>M-10</t>
+          <t>M-09</t>
         </is>
       </c>
       <c r="B75" s="4" t="inlineStr">
         <is>
-          <t>10 Encastre de fondo y zona de fondos (5 carros)</t>
+          <t>9 Soldadura longitudinal</t>
         </is>
       </c>
       <c r="C75" s="4" t="inlineStr">
@@ -4441,44 +4451,44 @@
         </is>
       </c>
       <c r="E75" s="5" t="n">
-        <v>21</v>
+        <v>23.4</v>
       </c>
       <c r="F75" s="5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G75" s="5" t="n">
-        <v>26.6</v>
+        <v>29.4</v>
       </c>
       <c r="H75" s="5" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I75" s="5" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="J75" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K75" s="5" t="n">
-        <v>22.4</v>
+        <v>24</v>
       </c>
       <c r="L75" s="5" t="n">
-        <v>3.6</v>
+        <v>8.4</v>
       </c>
       <c r="M75" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 3</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>M-11</t>
+          <t>M-PV</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>11 Bordoneado</t>
+          <t>Cuerpos soldados y cambio de formato</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -4492,44 +4502,46 @@
         </is>
       </c>
       <c r="E76" s="5" t="n">
-        <v>26.6</v>
+        <v>29.4</v>
       </c>
       <c r="F76" s="5" t="n">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G76" s="5" t="n">
-        <v>31</v>
+        <v>35.3</v>
       </c>
       <c r="H76" s="5" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="I76" s="5" t="n">
-        <v>4.4</v>
+        <v>5.9</v>
       </c>
       <c r="J76" s="5" t="n">
         <v>4</v>
       </c>
       <c r="K76" s="5" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="L76" s="5" t="n">
-        <v>3.6</v>
+        <v>23.6</v>
+      </c>
+      <c r="L76" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M76" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>W-MAN 7: PU-V2, PU-V3, PU-FX</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>M-PB</t>
+          <t>M-12</t>
         </is>
       </c>
       <c r="B77" s="4" t="inlineStr">
         <is>
-          <t>Pulmones del bordoneado a la soldadura circunferencial</t>
+          <t>12 Soldadura circunferencial (2 máquinas)</t>
         </is>
       </c>
       <c r="C77" s="4" t="inlineStr">
@@ -4543,46 +4555,44 @@
         </is>
       </c>
       <c r="E77" s="5" t="n">
-        <v>31</v>
+        <v>36.8</v>
       </c>
       <c r="F77" s="5" t="n">
-        <v>35</v>
+        <v>40.5</v>
       </c>
       <c r="G77" s="5" t="n">
-        <v>35.3</v>
+        <v>43.8</v>
       </c>
       <c r="H77" s="5" t="n">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="I77" s="5" t="n">
-        <v>4.3</v>
+        <v>7</v>
       </c>
       <c r="J77" s="5" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K77" s="5" t="n">
-        <v>17.2</v>
-      </c>
-      <c r="L77" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>31.5</v>
+      </c>
+      <c r="L77" s="5" t="n">
+        <v>17.5</v>
       </c>
       <c r="M77" s="4" t="inlineStr">
         <is>
-          <t>W-MAN 9 y 10</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>M-08</t>
+          <t>M-13</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>8 Cilindrado</t>
+          <t>13 Control de espesor</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -4596,44 +4606,44 @@
         </is>
       </c>
       <c r="E78" s="5" t="n">
-        <v>18</v>
+        <v>36.8</v>
       </c>
       <c r="F78" s="5" t="n">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="G78" s="5" t="n">
-        <v>23.4</v>
+        <v>43.8</v>
       </c>
       <c r="H78" s="5" t="n">
-        <v>33</v>
+        <v>40.5</v>
       </c>
       <c r="I78" s="5" t="n">
-        <v>5.4</v>
+        <v>7</v>
       </c>
       <c r="J78" s="5" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="K78" s="5" t="n">
-        <v>21.6</v>
+        <v>17.5</v>
       </c>
       <c r="L78" s="5" t="n">
-        <v>7.3</v>
+        <v>2.3</v>
       </c>
       <c r="M78" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 12: PU-S y 2 PU-RT</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>M-09</t>
+          <t>M-14</t>
         </is>
       </c>
       <c r="B79" s="4" t="inlineStr">
         <is>
-          <t>9 Soldadura longitudinal</t>
+          <t>14 Prueba hidráulica (2 bancos)</t>
         </is>
       </c>
       <c r="C79" s="4" t="inlineStr">
@@ -4647,44 +4657,44 @@
         </is>
       </c>
       <c r="E79" s="5" t="n">
-        <v>23.4</v>
+        <v>36.8</v>
       </c>
       <c r="F79" s="5" t="n">
-        <v>29</v>
+        <v>33.5</v>
       </c>
       <c r="G79" s="5" t="n">
-        <v>29.4</v>
+        <v>43.8</v>
       </c>
       <c r="H79" s="5" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="I79" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J79" s="5" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K79" s="5" t="n">
-        <v>24</v>
+        <v>31.5</v>
       </c>
       <c r="L79" s="5" t="n">
-        <v>8.4</v>
+        <v>14.1</v>
       </c>
       <c r="M79" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 13: 2 PU-6</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>M-PV</t>
+          <t>M-15</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>Cuerpos soldados y cambio de formato</t>
+          <t>15 Secado (4 secadoras)</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -4698,46 +4708,44 @@
         </is>
       </c>
       <c r="E80" s="5" t="n">
-        <v>29.4</v>
+        <v>36.8</v>
       </c>
       <c r="F80" s="5" t="n">
         <v>29</v>
       </c>
       <c r="G80" s="5" t="n">
-        <v>35.3</v>
+        <v>43.8</v>
       </c>
       <c r="H80" s="5" t="n">
-        <v>33</v>
+        <v>33.5</v>
       </c>
       <c r="I80" s="5" t="n">
-        <v>5.9</v>
+        <v>7</v>
       </c>
       <c r="J80" s="5" t="n">
-        <v>4</v>
+        <v>4.5</v>
       </c>
       <c r="K80" s="5" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="L80" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>31.5</v>
+      </c>
+      <c r="L80" s="5" t="n">
+        <v>6</v>
       </c>
       <c r="M80" s="4" t="inlineStr">
         <is>
-          <t>W-MAN 7: PU-V2, PU-V3, PU-FX</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 14: 2 PU-7</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>M-12</t>
+          <t>M-16</t>
         </is>
       </c>
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>12 Soldadura circunferencial (2 máquinas)</t>
+          <t>16 Granallado</t>
         </is>
       </c>
       <c r="C81" s="4" t="inlineStr">
@@ -4751,28 +4759,28 @@
         </is>
       </c>
       <c r="E81" s="5" t="n">
-        <v>36.8</v>
+        <v>45.3</v>
       </c>
       <c r="F81" s="5" t="n">
-        <v>40.5</v>
+        <v>29</v>
       </c>
       <c r="G81" s="5" t="n">
-        <v>43.8</v>
+        <v>51.8</v>
       </c>
       <c r="H81" s="5" t="n">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="I81" s="5" t="n">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="J81" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="K81" s="5" t="n">
-        <v>31.5</v>
+        <v>32.5</v>
       </c>
       <c r="L81" s="5" t="n">
-        <v>17.5</v>
+        <v>27.4</v>
       </c>
       <c r="M81" s="4" t="inlineStr">
         <is>
@@ -4783,12 +4791,12 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>M-13</t>
+          <t>M-17</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>13 Control de espesor</t>
+          <t>17 y 18 Detección y corrección de defectos</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -4802,44 +4810,44 @@
         </is>
       </c>
       <c r="E82" s="5" t="n">
-        <v>36.8</v>
+        <v>51.8</v>
       </c>
       <c r="F82" s="5" t="n">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="G82" s="5" t="n">
-        <v>43.8</v>
+        <v>57.3</v>
       </c>
       <c r="H82" s="5" t="n">
-        <v>40.5</v>
+        <v>34</v>
       </c>
       <c r="I82" s="5" t="n">
-        <v>7</v>
+        <v>5.5</v>
       </c>
       <c r="J82" s="5" t="n">
-        <v>2.5</v>
+        <v>5</v>
       </c>
       <c r="K82" s="5" t="n">
-        <v>17.5</v>
+        <v>27.5</v>
       </c>
       <c r="L82" s="5" t="n">
-        <v>2.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="M82" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 12: PU-S y 2 PU-RT</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 16 y 17 (3 jaulas y carro de corregibles)</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>M-14</t>
+          <t>M-18</t>
         </is>
       </c>
       <c r="B83" s="4" t="inlineStr">
         <is>
-          <t>14 Prueba hidráulica (2 bancos)</t>
+          <t>19 Cuelgue en el riel de la pintura</t>
         </is>
       </c>
       <c r="C83" s="4" t="inlineStr">
@@ -4853,49 +4861,51 @@
         </is>
       </c>
       <c r="E83" s="5" t="n">
-        <v>36.8</v>
+        <v>58.8</v>
       </c>
       <c r="F83" s="5" t="n">
-        <v>33.5</v>
+        <v>29</v>
       </c>
       <c r="G83" s="5" t="n">
-        <v>43.8</v>
+        <v>66</v>
       </c>
       <c r="H83" s="5" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I83" s="5" t="n">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="J83" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="K83" s="5" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="L83" s="5" t="n">
-        <v>14.1</v>
+        <v>36</v>
+      </c>
+      <c r="L83" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M83" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 13: 2 PU-6</t>
+          <t>W-MAN 18: carga de la línea; carros móviles y ganchos por formato</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>M-15</t>
+          <t>RV-M</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>15 Secado (4 secadoras)</t>
+          <t>Reserva de ampliación de manuales (junto a la columna de puestos saturados)</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>Manuales 1 a 10 kg</t>
+          <t>Libre / reserva</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -4904,49 +4914,51 @@
         </is>
       </c>
       <c r="E84" s="5" t="n">
-        <v>36.8</v>
+        <v>45.3</v>
       </c>
       <c r="F84" s="5" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G84" s="5" t="n">
-        <v>43.8</v>
+        <v>57.3</v>
       </c>
       <c r="H84" s="5" t="n">
-        <v>33.5</v>
+        <v>45</v>
       </c>
       <c r="I84" s="5" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="J84" s="5" t="n">
-        <v>4.5</v>
+        <v>11</v>
       </c>
       <c r="K84" s="5" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="L84" s="5" t="n">
-        <v>6</v>
+        <v>132</v>
+      </c>
+      <c r="L84" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M84" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 14: 2 PU-7</t>
+          <t>Lugar para la máquina siguiente de los puestos saturados en 2035. X-MAN 2035, aprovechamiento: sold. longitudinal 97 %, encastre, sold. circunferencial y prueba hidráulica 94 %, secado, preparación de cuello y etiquetado 92 %</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>M-16</t>
+          <t>RV-T</t>
         </is>
       </c>
       <c r="B85" s="4" t="inlineStr">
         <is>
-          <t>16 Granallado</t>
+          <t>Reserva de la pintura y del granallado</t>
         </is>
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>Manuales 1 a 10 kg</t>
+          <t>Libre / reserva</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -4955,49 +4967,51 @@
         </is>
       </c>
       <c r="E85" s="5" t="n">
-        <v>45.3</v>
+        <v>58.8</v>
       </c>
       <c r="F85" s="5" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="G85" s="5" t="n">
-        <v>51.8</v>
+        <v>66</v>
       </c>
       <c r="H85" s="5" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="I85" s="5" t="n">
-        <v>6.5</v>
+        <v>7.2</v>
       </c>
       <c r="J85" s="5" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="K85" s="5" t="n">
-        <v>32.5</v>
-      </c>
-      <c r="L85" s="5" t="n">
-        <v>27.4</v>
+        <v>79.2</v>
+      </c>
+      <c r="L85" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M85" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10</t>
+          <t>X-MAN 2035, aprovechamiento: sold. longitudinal 97 %, encastre, sold. circunferencial y prueba hidráulica 94 %, secado, preparación de cuello y etiquetado 92 %</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>M-17</t>
+          <t>M-19</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>17 y 18 Detección y corrección de defectos</t>
+          <t>19 Pintura en polvo + horno (línea Firesafer)</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>Manuales 1 a 10 kg</t>
+          <t>Pintura</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -5006,49 +5020,49 @@
         </is>
       </c>
       <c r="E86" s="5" t="n">
-        <v>51.8</v>
+        <v>66</v>
       </c>
       <c r="F86" s="5" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G86" s="5" t="n">
-        <v>57.3</v>
+        <v>76</v>
       </c>
       <c r="H86" s="5" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="I86" s="5" t="n">
-        <v>5.5</v>
+        <v>10</v>
       </c>
       <c r="J86" s="5" t="n">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="K86" s="5" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="L86" s="5" t="n">
-        <v>9.199999999999999</v>
+        <v>270</v>
+      </c>
+      <c r="L86" s="4" t="n">
+        <v>270</v>
       </c>
       <c r="M86" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10; W-MAN 16 y 17 (3 jaulas y carro de corregibles)</t>
+          <t>ET: 25000 × 8000 × 4000 mm; W-MAN 18 y X-MAN 19; franja de servicio de 1 m</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>M-18</t>
+          <t>M-20</t>
         </is>
       </c>
       <c r="B87" s="4" t="inlineStr">
         <is>
-          <t>19 Cuelgue en el riel de la pintura</t>
+          <t>20 a 25 Terminación: carga, ensamblaje, presurización, pérdidas, etiquetado y embalaje</t>
         </is>
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>Manuales 1 a 10 kg</t>
+          <t>Terminación de manuales</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -5060,48 +5074,46 @@
         <v>58.8</v>
       </c>
       <c r="F87" s="5" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="G87" s="5" t="n">
         <v>66</v>
       </c>
       <c r="H87" s="5" t="n">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="I87" s="5" t="n">
         <v>7.2</v>
       </c>
       <c r="J87" s="5" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="K87" s="5" t="n">
-        <v>36</v>
-      </c>
-      <c r="L87" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>64.8</v>
+      </c>
+      <c r="L87" s="5" t="n">
+        <v>47</v>
       </c>
       <c r="M87" s="4" t="inlineStr">
         <is>
-          <t>W-MAN 18: carga de la línea; carros móviles y ganchos por formato</t>
+          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10 (Guerchet de los puestos 20 a 25: 42,4 m² + 6 carros pulmón)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>RV-M</t>
+          <t>C-16</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Reserva de ampliación de manuales (junto a la columna de puestos saturados)</t>
+          <t>16 Depósito de PT de carros: retenidos (amarillo) y liberados (verde)</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>Libre / reserva</t>
+          <t>Depósitos de producto terminado</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -5110,46 +5122,44 @@
         </is>
       </c>
       <c r="E88" s="5" t="n">
-        <v>45.3</v>
+        <v>24.7</v>
       </c>
       <c r="F88" s="5" t="n">
-        <v>34</v>
+        <v>3.5</v>
       </c>
       <c r="G88" s="5" t="n">
-        <v>57.3</v>
+        <v>39.7</v>
       </c>
       <c r="H88" s="5" t="n">
-        <v>45</v>
+        <v>10.2</v>
       </c>
       <c r="I88" s="5" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J88" s="5" t="n">
-        <v>11</v>
+        <v>6.7</v>
       </c>
       <c r="K88" s="5" t="n">
-        <v>132</v>
-      </c>
-      <c r="L88" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>100.5</v>
+      </c>
+      <c r="L88" s="5" t="n">
+        <v>72</v>
       </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>Lugar para la máquina siguiente de los puestos saturados en 2035. X-MAN 2035, aprovechamiento: sold. longitudinal 97 %, encastre, sold. circunferencial y prueba hidráulica 94 %, secado, preparación de cuello y etiquetado 92 %</t>
+          <t>W-CAR, tabla de espacios del puesto 16: 0,5 m² por carro y los pasillos; 74 retenidos y 70 liberados (demanda 2035), paso de carros al norte</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>RV-T</t>
+          <t>RV-C1</t>
         </is>
       </c>
       <c r="B89" s="4" t="inlineStr">
         <is>
-          <t>Reserva de la pintura y del granallado</t>
+          <t>Libre (reserva del depósito de PT de carros)</t>
         </is>
       </c>
       <c r="C89" s="4" t="inlineStr">
@@ -5163,25 +5173,25 @@
         </is>
       </c>
       <c r="E89" s="5" t="n">
-        <v>58.8</v>
+        <v>24.7</v>
       </c>
       <c r="F89" s="5" t="n">
-        <v>34</v>
+        <v>10.2</v>
       </c>
       <c r="G89" s="5" t="n">
-        <v>66</v>
+        <v>37.7</v>
       </c>
       <c r="H89" s="5" t="n">
-        <v>45</v>
+        <v>13.5</v>
       </c>
       <c r="I89" s="5" t="n">
-        <v>7.2</v>
+        <v>13</v>
       </c>
       <c r="J89" s="5" t="n">
-        <v>11</v>
+        <v>3.3</v>
       </c>
       <c r="K89" s="5" t="n">
-        <v>79.2</v>
+        <v>42.9</v>
       </c>
       <c r="L89" s="4" t="inlineStr">
         <is>
@@ -5190,24 +5200,24 @@
       </c>
       <c r="M89" s="4" t="inlineStr">
         <is>
-          <t>X-MAN 2035, aprovechamiento: sold. longitudinal 97 %, encastre, sold. circunferencial y prueba hidráulica 94 %, secado, preparación de cuello y etiquetado 92 %</t>
+          <t>Lo que no ocupa la demanda 2035 en el depósito 16 (W-CAR pedía ≈ 200 m² para 20 carros por día)</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>M-19</t>
+          <t>C-16A</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>19 Pintura en polvo + horno (línea Firesafer)</t>
+          <t>16 Entrada de los cilindros pintados desde el pasillo principal</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>Pintura</t>
+          <t>Depósitos de producto terminado</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -5216,49 +5226,51 @@
         </is>
       </c>
       <c r="E90" s="5" t="n">
-        <v>66</v>
+        <v>37.7</v>
       </c>
       <c r="F90" s="5" t="n">
-        <v>20</v>
+        <v>10.2</v>
       </c>
       <c r="G90" s="5" t="n">
-        <v>76</v>
+        <v>39.7</v>
       </c>
       <c r="H90" s="5" t="n">
-        <v>47</v>
+        <v>13.5</v>
       </c>
       <c r="I90" s="5" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="J90" s="5" t="n">
-        <v>27</v>
+        <v>3.3</v>
       </c>
       <c r="K90" s="5" t="n">
-        <v>270</v>
-      </c>
-      <c r="L90" s="4" t="n">
-        <v>270</v>
+        <v>6.6</v>
+      </c>
+      <c r="L90" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>ET: 25000 × 8000 × 4000 mm; W-MAN 18 y X-MAN 19; franja de servicio de 1 m</t>
+          <t>Paso de carros a mano (criterio): los cilindros vendidos vacíos vienen del puesto 12 por C-11A y el pasillo principal</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>M-20</t>
+          <t>C-16P</t>
         </is>
       </c>
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>20 a 25 Terminación: carga, ensamblaje, presurización, pérdidas, etiquetado y embalaje</t>
+          <t>16 Pasillo de despacho (P2) y rechazados (rojo)</t>
         </is>
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>Terminación de manuales</t>
+          <t>Depósitos de producto terminado</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -5267,49 +5279,49 @@
         </is>
       </c>
       <c r="E91" s="5" t="n">
-        <v>58.8</v>
-      </c>
-      <c r="F91" s="5" t="n">
-        <v>20</v>
+        <v>24.7</v>
+      </c>
+      <c r="F91" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="G91" s="5" t="n">
-        <v>66</v>
+        <v>39.7</v>
       </c>
       <c r="H91" s="5" t="n">
-        <v>29</v>
+        <v>3.5</v>
       </c>
       <c r="I91" s="5" t="n">
-        <v>7.2</v>
+        <v>15</v>
       </c>
       <c r="J91" s="5" t="n">
-        <v>9</v>
+        <v>3.5</v>
       </c>
       <c r="K91" s="5" t="n">
-        <v>64.8</v>
+        <v>52.5</v>
       </c>
       <c r="L91" s="5" t="n">
-        <v>47</v>
+        <v>11.5</v>
       </c>
       <c r="M91" s="4" t="inlineStr">
         <is>
-          <t>W-MAN; máquina de X-MAN; medida de la tabla de áreas v10 (Guerchet de los puestos 20 a 25: 42,4 m² + 6 carros pulmón)</t>
+          <t>W-CAR 16: pasillo entre las zonas y la puerta; rechazados: 23 carros a 0,5 m²</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>C-16</t>
+          <t>C-17</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>16 Depósito de PT de carros: retenidos (amarillo) y liberados (verde)</t>
+          <t>17 Ensayos de lote (recinto de descarga, balanza y mesa)</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>Depósitos de producto terminado</t>
+          <t>Carros 25 a 100 kg</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -5318,95 +5330,95 @@
         </is>
       </c>
       <c r="E92" s="5" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="F92" s="5" t="n">
-        <v>3.5</v>
+        <v>39.7</v>
+      </c>
+      <c r="F92" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="G92" s="5" t="n">
-        <v>39.7</v>
+        <v>55.2</v>
       </c>
       <c r="H92" s="5" t="n">
-        <v>13.5</v>
+        <v>4.5</v>
       </c>
       <c r="I92" s="5" t="n">
-        <v>15</v>
+        <v>15.5</v>
       </c>
       <c r="J92" s="5" t="n">
-        <v>10</v>
+        <v>4.5</v>
       </c>
       <c r="K92" s="5" t="n">
-        <v>150</v>
+        <v>69.75</v>
       </c>
       <c r="L92" s="4" t="n">
-        <v>150</v>
+        <v>70</v>
       </c>
       <c r="M92" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 16: retenidos ≈ 9 × 10 m (180 carros), liberados ≈ 6 × 10 m (100 carros), pasillo hasta la puerta</t>
+          <t>W-CAR, tabla de espacios del puesto 17: ≈ 15,5 × 4,5 m (el patio de rodadura va afuera)</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>C-16P</t>
+          <t>C-14</t>
         </is>
       </c>
       <c r="B93" s="4" t="inlineStr">
         <is>
-          <t>16 Pasillo de despacho (P2) y rechazados (rojo)</t>
+          <t>14 Sala del ensayo de pérdidas (paneles aislantes, split)</t>
         </is>
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>Depósitos de producto terminado</t>
+          <t>Carros 25 a 100 kg</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>local</t>
         </is>
       </c>
       <c r="E93" s="5" t="n">
-        <v>24.7</v>
-      </c>
-      <c r="F93" s="4" t="n">
-        <v>0</v>
+        <v>39.7</v>
+      </c>
+      <c r="F93" s="5" t="n">
+        <v>4.5</v>
       </c>
       <c r="G93" s="5" t="n">
-        <v>39.7</v>
+        <v>43.7</v>
       </c>
       <c r="H93" s="5" t="n">
-        <v>3.5</v>
+        <v>8.5</v>
       </c>
       <c r="I93" s="5" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="J93" s="5" t="n">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="K93" s="5" t="n">
-        <v>52.5</v>
-      </c>
-      <c r="L93" s="4" t="n">
-        <v>50</v>
+        <v>16</v>
+      </c>
+      <c r="L93" s="5" t="n">
+        <v>14.16666666666667</v>
       </c>
       <c r="M93" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: pasillo del autoelevador entre las zonas y la puerta; rechazados ≈ 5 × 3 m</t>
+          <t>W-CAR 14: 25 m² para 30 lugares; con los 17 de 2035, a la misma relación</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>C-17</t>
+          <t>C-15</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>17 Ensayos de lote (recinto de descarga, balanza y mesa)</t>
+          <t>15 Etiquetado e inspección final</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -5422,42 +5434,42 @@
       <c r="E94" s="5" t="n">
         <v>39.7</v>
       </c>
-      <c r="F94" s="4" t="n">
-        <v>0</v>
+      <c r="F94" s="5" t="n">
+        <v>8.5</v>
       </c>
       <c r="G94" s="5" t="n">
-        <v>55.2</v>
+        <v>43.7</v>
       </c>
       <c r="H94" s="5" t="n">
-        <v>4.5</v>
+        <v>13.5</v>
       </c>
       <c r="I94" s="5" t="n">
-        <v>15.5</v>
+        <v>4</v>
       </c>
       <c r="J94" s="5" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="K94" s="5" t="n">
-        <v>69.75</v>
+        <v>20</v>
       </c>
       <c r="L94" s="4" t="n">
-        <v>70</v>
+        <v>9</v>
       </c>
       <c r="M94" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 17: ≈ 15,5 × 4,5 m (el patio de rodadura va afuera)</t>
+          <t>W-CAR, tabla de espacios del puesto 15: ≈ 3,5 × 2,5 m, más el paso de los carros al depósito 16</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>C-14</t>
+          <t>C-13</t>
         </is>
       </c>
       <c r="B95" s="4" t="inlineStr">
         <is>
-          <t>14 Sala del ensayo de pérdidas (paneles aislantes, split)</t>
+          <t>13 Carga, armado y presurización</t>
         </is>
       </c>
       <c r="C95" s="4" t="inlineStr">
@@ -5467,48 +5479,48 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>local</t>
+          <t>area</t>
         </is>
       </c>
       <c r="E95" s="5" t="n">
-        <v>39.7</v>
+        <v>43.7</v>
       </c>
       <c r="F95" s="5" t="n">
-        <v>4.5</v>
+        <v>7</v>
       </c>
       <c r="G95" s="5" t="n">
-        <v>44.7</v>
+        <v>55.2</v>
       </c>
       <c r="H95" s="5" t="n">
-        <v>9.5</v>
+        <v>13.5</v>
       </c>
       <c r="I95" s="5" t="n">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="J95" s="5" t="n">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="K95" s="5" t="n">
-        <v>25</v>
+        <v>74.75</v>
       </c>
       <c r="L95" s="4" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="M95" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 14: 5,0 × 5,0 m, 30 lugares numerados</t>
+          <t>W-CAR, tabla de espacios del puesto 13: ≈ 10 × 6 m</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>C-15</t>
+          <t>C-1314</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>15 Etiquetado e inspección final</t>
+          <t>Paso de la carga a la sala de pérdidas y a los ensayos</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -5522,44 +5534,46 @@
         </is>
       </c>
       <c r="E96" s="5" t="n">
-        <v>39.7</v>
+        <v>43.7</v>
       </c>
       <c r="F96" s="5" t="n">
-        <v>9.5</v>
+        <v>4.5</v>
       </c>
       <c r="G96" s="5" t="n">
-        <v>44.7</v>
+        <v>55.2</v>
       </c>
       <c r="H96" s="5" t="n">
-        <v>13.5</v>
+        <v>7</v>
       </c>
       <c r="I96" s="5" t="n">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="J96" s="5" t="n">
-        <v>4</v>
+        <v>2.5</v>
       </c>
       <c r="K96" s="5" t="n">
-        <v>20</v>
-      </c>
-      <c r="L96" s="4" t="n">
-        <v>9</v>
+        <v>28.75</v>
+      </c>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M96" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 15: ≈ 3,5 × 2,5 m, más el paso de los carros al depósito 16</t>
+          <t>W-CAR 13, 14 y 17: recorrido de los carros de la muestra; estanterías del puesto 13</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>C-13</t>
+          <t>C-12</t>
         </is>
       </c>
       <c r="B97" s="4" t="inlineStr">
         <is>
-          <t>13 Carga, armado y presurización</t>
+          <t>12 Pulmón de pintados (49 carros), al lado del puesto 13</t>
         </is>
       </c>
       <c r="C97" s="4" t="inlineStr">
@@ -5573,49 +5587,49 @@
         </is>
       </c>
       <c r="E97" s="5" t="n">
-        <v>44.7</v>
+        <v>55.2</v>
       </c>
       <c r="F97" s="5" t="n">
-        <v>7</v>
+        <v>3.3</v>
       </c>
       <c r="G97" s="5" t="n">
-        <v>55.2</v>
+        <v>61.40000000000001</v>
       </c>
       <c r="H97" s="5" t="n">
-        <v>13.5</v>
+        <v>8.6</v>
       </c>
       <c r="I97" s="5" t="n">
-        <v>10.5</v>
+        <v>6.2</v>
       </c>
       <c r="J97" s="5" t="n">
-        <v>6.5</v>
+        <v>5.3</v>
       </c>
       <c r="K97" s="5" t="n">
-        <v>68.25</v>
-      </c>
-      <c r="L97" s="4" t="n">
-        <v>60</v>
+        <v>32.86</v>
+      </c>
+      <c r="L97" s="5" t="n">
+        <v>24.5</v>
       </c>
       <c r="M97" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 13: ≈ 10 × 6 m</t>
+          <t>W-CAR 12: filas por modelo y lote, al lado del puesto 13; 49 carros a 0,5 m²</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>C-1314</t>
+          <t>RV-C2</t>
         </is>
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>Paso de la carga a la sala de pérdidas y a los ensayos</t>
+          <t>Libre (reserva del pulmón de pintados)</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Libre / reserva</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -5624,25 +5638,25 @@
         </is>
       </c>
       <c r="E98" s="5" t="n">
-        <v>44.7</v>
+        <v>55.2</v>
       </c>
       <c r="F98" s="5" t="n">
-        <v>4.5</v>
+        <v>8.6</v>
       </c>
       <c r="G98" s="5" t="n">
-        <v>55.2</v>
+        <v>61.40000000000001</v>
       </c>
       <c r="H98" s="5" t="n">
-        <v>7</v>
+        <v>13.5</v>
       </c>
       <c r="I98" s="5" t="n">
-        <v>10.5</v>
+        <v>6.2</v>
       </c>
       <c r="J98" s="5" t="n">
-        <v>2.5</v>
+        <v>4.9</v>
       </c>
       <c r="K98" s="5" t="n">
-        <v>26.25</v>
+        <v>30.38</v>
       </c>
       <c r="L98" s="4" t="inlineStr">
         <is>
@@ -5651,19 +5665,19 @@
       </c>
       <c r="M98" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 13, 14 y 17: recorrido de los carros de la muestra; estanterías del puesto 13</t>
+          <t>Lo que no ocupa la demanda 2035 en el pulmón 12 (W-CAR: 120 carros para 20 por día)</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>C-12</t>
+          <t>C-12C</t>
         </is>
       </c>
       <c r="B99" s="4" t="inlineStr">
         <is>
-          <t>12 Pulmón de pintados (120 carros), al lado del puesto 13</t>
+          <t>12 Recepción de pintados: cambio de juego y rechazados del pintor (P6)</t>
         </is>
       </c>
       <c r="C99" s="4" t="inlineStr">
@@ -5679,23 +5693,23 @@
       <c r="E99" s="5" t="n">
         <v>55.2</v>
       </c>
-      <c r="F99" s="5" t="n">
-        <v>3.3</v>
+      <c r="F99" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="G99" s="5" t="n">
         <v>61.40000000000001</v>
       </c>
       <c r="H99" s="5" t="n">
-        <v>13.5</v>
+        <v>3.3</v>
       </c>
       <c r="I99" s="5" t="n">
         <v>6.2</v>
       </c>
       <c r="J99" s="5" t="n">
-        <v>10.2</v>
+        <v>3.3</v>
       </c>
       <c r="K99" s="5" t="n">
-        <v>63.24</v>
+        <v>20.46</v>
       </c>
       <c r="L99" s="4" t="inlineStr">
         <is>
@@ -5704,19 +5718,19 @@
       </c>
       <c r="M99" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 12: pulmón de pintados ≈ 10 × 7 m, filas por modelo y lote; el puesto 12 (con C-12C) ≈ 79 m²</t>
+          <t>W-CAR 12: 2 lugares de cambio de juego de 2,0 × 1,5 m y rechazados ≈ 2 × 1,5 m, al lado de la puerta</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>C-12C</t>
+          <t>C-11A</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>12 Recepción de pintados: cambio de juego y rechazados del pintor (P6)</t>
+          <t>11 Pasillo de los carros a la puerta (secos, cilindros pintados)</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -5730,25 +5744,25 @@
         </is>
       </c>
       <c r="E100" s="5" t="n">
-        <v>55.2</v>
-      </c>
-      <c r="F100" s="4" t="n">
-        <v>0</v>
+        <v>61.40000000000001</v>
+      </c>
+      <c r="F100" s="5" t="n">
+        <v>2.25</v>
       </c>
       <c r="G100" s="5" t="n">
-        <v>61.40000000000001</v>
+        <v>62.40000000000001</v>
       </c>
       <c r="H100" s="5" t="n">
-        <v>3.3</v>
+        <v>13.5</v>
       </c>
       <c r="I100" s="5" t="n">
-        <v>6.2</v>
+        <v>1</v>
       </c>
       <c r="J100" s="5" t="n">
-        <v>3.3</v>
+        <v>11.25</v>
       </c>
       <c r="K100" s="5" t="n">
-        <v>20.46</v>
+        <v>11.25</v>
       </c>
       <c r="L100" s="4" t="inlineStr">
         <is>
@@ -5757,19 +5771,19 @@
       </c>
       <c r="M100" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 12: 2 lugares de cambio de juego de 2,0 × 1,5 m y rechazados ≈ 2 × 1,5 m, al lado de la puerta</t>
+          <t>W-CAR 11: pasillo ≈ 1 m entre las filas y la puerta; por acá suben los cilindros pintados al pasillo principal</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>C-11A</t>
+          <t>C-11</t>
         </is>
       </c>
       <c r="B101" s="4" t="inlineStr">
         <is>
-          <t>11 Pasillo de los carros a la puerta</t>
+          <t>11 Pulmón de despacho a la pintura tercerizada (84 carros)</t>
         </is>
       </c>
       <c r="C101" s="4" t="inlineStr">
@@ -5783,51 +5797,49 @@
         </is>
       </c>
       <c r="E101" s="5" t="n">
-        <v>61.40000000000001</v>
+        <v>62.40000000000001</v>
       </c>
       <c r="F101" s="5" t="n">
         <v>2.25</v>
       </c>
       <c r="G101" s="5" t="n">
-        <v>62.40000000000001</v>
+        <v>67.59999999999999</v>
       </c>
       <c r="H101" s="5" t="n">
-        <v>13.5</v>
+        <v>10.7</v>
       </c>
       <c r="I101" s="5" t="n">
-        <v>1</v>
+        <v>5.2</v>
       </c>
       <c r="J101" s="5" t="n">
-        <v>11.25</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="K101" s="5" t="n">
-        <v>11.25</v>
-      </c>
-      <c r="L101" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>43.94</v>
+      </c>
+      <c r="L101" s="5" t="n">
+        <v>42</v>
       </c>
       <c r="M101" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 11: pasillo ≈ 10 × 1 m entre las filas y la puerta</t>
+          <t>W-CAR, tabla de espacios del puesto 11: filas por modelo y semana, demarcadas en amarillo; 84 carros a 0,5 m²</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>C-11</t>
+          <t>RV-C3</t>
         </is>
       </c>
       <c r="B102" s="4" t="inlineStr">
         <is>
-          <t>11 Pulmón de despacho a la pintura tercerizada (120 carros)</t>
+          <t>Libre (reserva del pulmón de despacho)</t>
         </is>
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>Carros 25 a 100 kg</t>
+          <t>Libre / reserva</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -5839,7 +5851,7 @@
         <v>62.40000000000001</v>
       </c>
       <c r="F102" s="5" t="n">
-        <v>2.25</v>
+        <v>10.7</v>
       </c>
       <c r="G102" s="5" t="n">
         <v>67.59999999999999</v>
@@ -5851,17 +5863,19 @@
         <v>5.2</v>
       </c>
       <c r="J102" s="5" t="n">
-        <v>11.25</v>
+        <v>2.8</v>
       </c>
       <c r="K102" s="5" t="n">
-        <v>58.5</v>
-      </c>
-      <c r="L102" s="4" t="n">
-        <v>57</v>
+        <v>14.56</v>
+      </c>
+      <c r="L102" s="4" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="M102" s="4" t="inlineStr">
         <is>
-          <t>W-CAR, tabla de espacios del puesto 11: filas por modelo y semana ≈ 10 × 6 m, demarcadas en amarillo</t>
+          <t>Lo que no ocupa la demanda 2035 en el pulmón 11 (W-CAR: 120 carros para 20 por día)</t>
         </is>
       </c>
     </row>
@@ -19227,7 +19241,7 @@
       </c>
       <c r="B219" s="4" t="inlineStr">
         <is>
-          <t>Pulmón de despacho: 15 filas de 8 carros por modelo y semana (120)</t>
+          <t>Pulmón de despacho: 11 filas de 8 carros por modelo y semana (84)</t>
         </is>
       </c>
       <c r="C219" s="4" t="inlineStr">
@@ -19244,19 +19258,19 @@
         <v>62.45</v>
       </c>
       <c r="F219" s="5" t="n">
-        <v>2.35</v>
+        <v>2.4</v>
       </c>
       <c r="G219" s="5" t="n">
         <v>67.55</v>
       </c>
       <c r="H219" s="5" t="n">
-        <v>12.75</v>
+        <v>10.1</v>
       </c>
       <c r="I219" s="5" t="n">
         <v>5.1</v>
       </c>
       <c r="J219" s="5" t="n">
-        <v>10.4</v>
+        <v>7.7</v>
       </c>
       <c r="K219" s="4" t="inlineStr">
         <is>
@@ -19269,7 +19283,7 @@
       <c r="M219" s="4" t="inlineStr"/>
       <c r="N219" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 11: 120 carros ≈ 10 × 6 m</t>
+          <t>W-CAR 11 con la demanda 2035: 84 carros</t>
         </is>
       </c>
     </row>
@@ -19335,7 +19349,7 @@
       </c>
       <c r="B221" s="4" t="inlineStr">
         <is>
-          <t>Pulmón de pintados: 15 filas de 8 carros por modelo y lote (120)</t>
+          <t>Pulmón de pintados: 7 filas de 7 carros por modelo y lote (49)</t>
         </is>
       </c>
       <c r="C221" s="4" t="inlineStr">
@@ -19355,16 +19369,16 @@
         <v>3.45</v>
       </c>
       <c r="G221" s="5" t="n">
-        <v>60.35</v>
+        <v>59.75</v>
       </c>
       <c r="H221" s="5" t="n">
-        <v>12.75</v>
+        <v>8.35</v>
       </c>
       <c r="I221" s="5" t="n">
-        <v>5.1</v>
+        <v>4.5</v>
       </c>
       <c r="J221" s="5" t="n">
-        <v>9.300000000000001</v>
+        <v>4.9</v>
       </c>
       <c r="K221" s="4" t="inlineStr">
         <is>
@@ -19377,7 +19391,7 @@
       <c r="M221" s="4" t="inlineStr"/>
       <c r="N221" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 12: 120 carros ≈ 10 × 7 m, al lado del puesto 13</t>
+          <t>W-CAR 12 con la demanda 2035: 49 carros</t>
         </is>
       </c>
     </row>
@@ -19933,7 +19947,7 @@
       </c>
       <c r="B232" s="4" t="inlineStr">
         <is>
-          <t>Muestra: lugares 1 a 16</t>
+          <t>Muestra: lugares 1 a 6</t>
         </is>
       </c>
       <c r="C232" s="4" t="inlineStr">
@@ -19950,19 +19964,19 @@
         <v>39.85</v>
       </c>
       <c r="F232" s="5" t="n">
-        <v>7.6</v>
+        <v>4.6</v>
       </c>
       <c r="G232" s="5" t="n">
-        <v>43.85</v>
+        <v>43.55</v>
       </c>
       <c r="H232" s="5" t="n">
-        <v>9</v>
+        <v>5.3</v>
       </c>
       <c r="I232" s="5" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="J232" s="5" t="n">
-        <v>1.4</v>
+        <v>0.7</v>
       </c>
       <c r="K232" s="4" t="inlineStr">
         <is>
@@ -19975,7 +19989,7 @@
       <c r="M232" s="4" t="inlineStr"/>
       <c r="N232" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 14: 30 lugares de 0,5 m²</t>
+          <t>W-CAR 14 con la muestra de 2035: 17 lugares de 0,5 m²</t>
         </is>
       </c>
     </row>
@@ -19987,7 +20001,7 @@
       </c>
       <c r="B233" s="4" t="inlineStr">
         <is>
-          <t>Muestra: lugares 17 a 30</t>
+          <t>Muestra: lugares 7 a 17</t>
         </is>
       </c>
       <c r="C233" s="4" t="inlineStr">
@@ -20004,16 +20018,16 @@
         <v>39.85</v>
       </c>
       <c r="F233" s="5" t="n">
-        <v>4.6</v>
+        <v>6.2</v>
       </c>
       <c r="G233" s="5" t="n">
-        <v>43.85</v>
+        <v>43.55</v>
       </c>
       <c r="H233" s="5" t="n">
-        <v>6</v>
+        <v>7.6</v>
       </c>
       <c r="I233" s="5" t="n">
-        <v>4</v>
+        <v>3.7</v>
       </c>
       <c r="J233" s="5" t="n">
         <v>1.4</v>
@@ -20029,7 +20043,7 @@
       <c r="M233" s="4" t="inlineStr"/>
       <c r="N233" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 14: 30 lugares de 0,5 m²</t>
+          <t>W-CAR 14 con la muestra de 2035: 17 lugares de 0,5 m²</t>
         </is>
       </c>
     </row>
@@ -20058,19 +20072,19 @@
         <v>39.75</v>
       </c>
       <c r="F234" s="5" t="n">
-        <v>6.3</v>
+        <v>5.35</v>
       </c>
       <c r="G234" s="5" t="n">
         <v>40</v>
       </c>
       <c r="H234" s="5" t="n">
-        <v>7.4</v>
+        <v>6.15</v>
       </c>
       <c r="I234" s="5" t="n">
         <v>0.25</v>
       </c>
       <c r="J234" s="5" t="n">
-        <v>1.1</v>
+        <v>0.8</v>
       </c>
       <c r="K234" s="4" t="inlineStr">
         <is>
@@ -20109,16 +20123,16 @@
         </is>
       </c>
       <c r="E235" s="5" t="n">
-        <v>42.4</v>
+        <v>41.5</v>
       </c>
       <c r="F235" s="5" t="n">
-        <v>10.6</v>
+        <v>10.9</v>
       </c>
       <c r="G235" s="5" t="n">
-        <v>44.4</v>
+        <v>43.5</v>
       </c>
       <c r="H235" s="5" t="n">
-        <v>11.4</v>
+        <v>11.7</v>
       </c>
       <c r="I235" s="5" t="n">
         <v>2</v>
@@ -20163,16 +20177,16 @@
         </is>
       </c>
       <c r="E236" s="5" t="n">
-        <v>40.8</v>
+        <v>40.1</v>
       </c>
       <c r="F236" s="5" t="n">
-        <v>10.7</v>
+        <v>11</v>
       </c>
       <c r="G236" s="5" t="n">
-        <v>42</v>
+        <v>41.3</v>
       </c>
       <c r="H236" s="5" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="I236" s="5" t="n">
         <v>1.2</v>
@@ -20217,16 +20231,16 @@
         </is>
       </c>
       <c r="E237" s="5" t="n">
-        <v>39.9</v>
+        <v>42</v>
       </c>
       <c r="F237" s="5" t="n">
-        <v>9.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="G237" s="5" t="n">
-        <v>41.4</v>
+        <v>43.5</v>
       </c>
       <c r="H237" s="5" t="n">
-        <v>10.6</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="I237" s="5" t="n">
         <v>1.5</v>
@@ -20257,7 +20271,7 @@
       </c>
       <c r="B238" s="4" t="inlineStr">
         <is>
-          <t>Liberados: 10 filas de 10 carros (100)</t>
+          <t>Liberados: 9 filas de 8 carros (70)</t>
         </is>
       </c>
       <c r="C238" s="4" t="inlineStr">
@@ -20271,22 +20285,22 @@
         </is>
       </c>
       <c r="E238" s="5" t="n">
-        <v>24.75</v>
+        <v>24.85</v>
       </c>
       <c r="F238" s="5" t="n">
         <v>3.6</v>
       </c>
       <c r="G238" s="5" t="n">
-        <v>30.65</v>
+        <v>31.15</v>
       </c>
       <c r="H238" s="5" t="n">
-        <v>12.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I238" s="5" t="n">
-        <v>5.9</v>
+        <v>6.3</v>
       </c>
       <c r="J238" s="5" t="n">
-        <v>9</v>
+        <v>5.1</v>
       </c>
       <c r="K238" s="4" t="inlineStr">
         <is>
@@ -20299,7 +20313,7 @@
       <c r="M238" s="4" t="inlineStr"/>
       <c r="N238" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: una semana de producción, ≈ 6 × 10 m</t>
+          <t>W-CAR 16 con la demanda 2035: una semana, 70 carros</t>
         </is>
       </c>
     </row>
@@ -20311,7 +20325,7 @@
       </c>
       <c r="B239" s="4" t="inlineStr">
         <is>
-          <t>Retenidos: 15 filas de 12 carros (180)</t>
+          <t>Retenidos: 10 filas de 8 carros (74)</t>
         </is>
       </c>
       <c r="C239" s="4" t="inlineStr">
@@ -20325,22 +20339,22 @@
         </is>
       </c>
       <c r="E239" s="5" t="n">
-        <v>30.75</v>
+        <v>31.95</v>
       </c>
       <c r="F239" s="5" t="n">
         <v>3.6</v>
       </c>
       <c r="G239" s="5" t="n">
-        <v>39.65</v>
+        <v>38.95</v>
       </c>
       <c r="H239" s="5" t="n">
-        <v>12.6</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="I239" s="5" t="n">
-        <v>8.9</v>
+        <v>7</v>
       </c>
       <c r="J239" s="5" t="n">
-        <v>9</v>
+        <v>5.1</v>
       </c>
       <c r="K239" s="4" t="inlineStr">
         <is>
@@ -20353,7 +20367,7 @@
       <c r="M239" s="4" t="inlineStr"/>
       <c r="N239" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: hasta 180 carros, ≈ 9 × 10 m</t>
+          <t>W-CAR 16 con la demanda 2035: 1,8 semanas de matafuegos, 74 carros</t>
         </is>
       </c>
     </row>
@@ -20419,7 +20433,7 @@
       </c>
       <c r="B241" s="4" t="inlineStr">
         <is>
-          <t>Zona de rechazados (roja)</t>
+          <t>Zona de rechazados (roja): 23 carros</t>
         </is>
       </c>
       <c r="C241" s="4" t="inlineStr">
@@ -20433,19 +20447,19 @@
         </is>
       </c>
       <c r="E241" s="5" t="n">
-        <v>34.6</v>
+        <v>35.6</v>
       </c>
       <c r="F241" s="5" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="G241" s="5" t="n">
         <v>39.6</v>
       </c>
       <c r="H241" s="5" t="n">
-        <v>3.25</v>
+        <v>3.3</v>
       </c>
       <c r="I241" s="5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J241" s="5" t="n">
         <v>3</v>
@@ -20461,7 +20475,7 @@
       <c r="M241" s="4" t="inlineStr"/>
       <c r="N241" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: ≈ 5 × 3 m</t>
+          <t>W-CAR 16: el lote de 50 kg de 2035 a 0,5 m², 4 × 3 m</t>
         </is>
       </c>
     </row>
@@ -20829,7 +20843,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cantidades del Word de carros (W-CAR, tablas de espacios de los puestos 11, 12, 14 y 16).</t>
+          <t>Reglas del Word de carros (W-CAR, puestos 11, 12, 14 y 16) aplicadas al mes pico de 2035 (X-CAR, Plan mensual): 69,8 recipientes por semana (40,8 matafuegos y 29,0 cilindros vendidos vacíos), 14,0 por día.</t>
         </is>
       </c>
     </row>
@@ -20851,12 +20865,12 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Criterio de W-CAR</t>
+          <t>Regla de W-CAR aplicada a 2035</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>Medida de W-CAR</t>
+          <t>Medida en planta</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -20883,16 +20897,16 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 11: hasta 100 carros (una semana) más los que se hacen mientras se espera el camión</t>
+          <t>W-CAR 11: 1 semana + 1 día de espera del camión (100 + 20 en el Word). 2035: 69,8 + 14,0 (entran en 1 semirremolque)</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>≈ 10 × 6 m</t>
+          <t>5,1 × 7,7 m</t>
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>120</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6">
@@ -20913,16 +20927,16 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 12: el mismo tamaño que el pulmón de despacho, al lado del puesto 13</t>
+          <t>W-CAR 12: como el 11 (1 semana + 1 día), sólo lo que va al 13 (los cilindros vacíos van a liberados). 2035: 40,8 × 1,2</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>≈ 10 × 7 m</t>
+          <t>4,5 × 4,9 m</t>
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>120</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7">
@@ -20943,16 +20957,16 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 14: unos 25 por semana durante 7 días, más los que esperan el puesto 17</t>
+          <t>W-CAR 14: muestra de la tabla del Word con los lotes de 2035 (3 + 8 + 1,5 + 1,5 = 14,0 por semana) × 30 / 25</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>5,0 × 5,0 m</t>
+          <t>4,0 × 4,0 m</t>
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -20973,16 +20987,16 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: el lote de una semana se libera al final de la siguiente: hasta unos 180 carros</t>
+          <t>W-CAR 16: el lote de la semana y casi todo el siguiente (180 = 1,8 semanas en el Word). 2035: 1,8 × 40,8 matafuegos</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>≈ 9 × 10 m</t>
+          <t>7,0 × 5,1 m</t>
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>180</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -20998,21 +21012,21 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Lotes liberados hasta el despacho</t>
+          <t>Lotes liberados y cilindros vendidos vacíos hasta el despacho</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: una semana de producción, unos 100 carros</t>
+          <t>W-CAR 16: una semana de producción (matafuegos y cilindros vendidos vacíos). 2035: 69,8</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>≈ 6 × 10 m</t>
+          <t>6,3 × 5,1 m</t>
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>100</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10">
@@ -21033,18 +21047,16 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>W-CAR 16: zona chica, casi nunca se usa</t>
+          <t>W-CAR 16: el lote rechazado entero; el mayor de 2035 es el de 50 kg (22,4 por semana)</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>≈ 5 × 3 m</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+          <t>4,0 × 3,0 m</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>